<commit_message>
Earnings models: no neutral defaults (exclude missing + rescale to 100, show Data coverage %), BMO/AMC timing scored, UW analyst ratings, Finnhub guidance hit-rate, drop Sloan, VIX proxy
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data_Health_Check.xlsx
+++ b/Data_Health_Check.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,11 +52,6 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -70,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -80,9 +75,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -669,7 +661,7 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 125 rows; {"source": "company", "report_time": "postmarket", "expected_move_perc": "0.04038960288808664260", "</t>
+          <t>AAPL: 125 rows; {"source": "company", "report_date": "2026-11-02", "report_time": "postmarket", "ending_fiscal_quart</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -755,7 +747,7 @@
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AAPL: {"last_trade": {"price": "346.2", "time": 1792686113532, "vol": 15065627}, "market_time": "regular", "quote": </t>
+          <t>AAPL: {"last_trade": {"price": "345.656", "time": 1792687345905, "vol": 15970483}, "market_time": "regular", "quote"</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -798,7 +790,7 @@
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"last_trade": {"price": "765.7", "time": 1792686119402, "vol": 19515027}, "market_time": "regular", "quote": </t>
+          <t>{"last_trade": {"price": "763.32", "time": 1792687350082, "vol": 20547728}, "market_time": "regular", "quote":</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -815,7 +807,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>VIX regime</t>
+          <t>VIX index (raw endpoint)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -858,7 +850,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Market tide (market flow)</t>
+          <t>VIX regime proxy (VIXY ETF quote)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -868,7 +860,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>/api/market/market-tide</t>
+          <t>/api/stock/VIXY/quote</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -884,12 +876,12 @@
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>58 rows; {"timestamp": "2026-10-22T07:30:00-04:00", "date": "2026-10-22", "net_call_premium": "-31513.0000", "</t>
+          <t>{"last_trade": {"price": "17.5183", "time": 1792687345664, "vol": 3180656}, "market_time": "regular", "quote":</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Pre-Earnings Direction, Unusual Activity</t>
+          <t>Kimi, Claude Pro</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -901,7 +893,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Options flow / sweeps</t>
+          <t>Market tide (market flow)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -911,7 +903,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/flow-alerts?limit</t>
+          <t>/api/market/market-tide</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -927,24 +919,24 @@
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 50 rows; {"type": "put", "ticker": "AAPL", "iv": 0.2973627839569233, "created_at": "2026-10-22T16:21:33.117498</t>
+          <t>62 rows; {"timestamp": "2026-10-22T07:30:00-04:00", "date": "2026-10-22", "net_call_premium": "-31513.0000", "</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
+          <t>Pre-Earnings Direction, Unusual Activity</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>7/7</t>
+          <t>1/1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Unusual options activity</t>
+          <t>Options flow / sweeps</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -954,7 +946,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>/api/option-activity/unusual?ticker_symbol&amp;min_premium&amp;limit&amp;unusual</t>
+          <t>/api/stock/{t}/flow-alerts?limit</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -970,12 +962,12 @@
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 13 rows; {"theta": "-0.910654120882431", "cross_volume": 0, "delta": "-0.404521796784856", "ticker_symbol": "A</t>
+          <t>AAPL: 50 rows; {"type": "put", "ticker": "AAPL", "iv": 0.31790407450507946, "created_at": "2026-10-22T16:42:20.70368</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction, Unusual Activity</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -987,7 +979,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>OI positioning / OI change</t>
+          <t>Unusual options activity</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -997,7 +989,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/oi-change?limit</t>
+          <t>/api/option-activity/unusual?ticker_symbol&amp;min_premium&amp;limit&amp;unusual</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1013,12 +1005,12 @@
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 100 rows; {"trades": 304, "volume": 18094, "option_symbol": "AAPL261218P00315000", "underlying_symbol": "AAPL"</t>
+          <t>AAPL: 12 rows; {"theta": "-0.945558737799859", "cross_volume": 0, "delta": "-0.4455248061730525", "ticker_symbol": "</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction, Unusual Activity</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1030,7 +1022,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Options volume / put-call</t>
+          <t>OI positioning / OI change</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1040,7 +1032,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/options-volume</t>
+          <t>/api/stock/{t}/oi-change?limit</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1056,12 +1048,12 @@
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 1 rows; {"date": "2026-10-22", "call_volume": 329695, "put_volume": 281087, "call_volume_ask_side": 144930, "c</t>
+          <t>AAPL: 100 rows; {"trades": 304, "volume": 18094, "option_symbol": "AAPL261218P00315000", "underlying_symbol": "AAPL"</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Unusual Activity</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1073,7 +1065,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Net premium ticks (call/put premium)</t>
+          <t>Options volume / put-call</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1083,7 +1075,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/net-prem-ticks</t>
+          <t>/api/stock/{t}/options-volume</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1099,12 +1091,12 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 228 rows; {"date": "2026-10-22", "call_volume": 3, "put_volume": 1, "call_volume_ask_side": 0, "call_volume_bi</t>
+          <t>AAPL: 1 rows; {"date": "2026-10-22", "call_volume": 354339, "put_volume": 304365, "call_volume_ask_side": 155182, "c</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Claude, Meta, Unusual Activity</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Unusual Activity</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1116,7 +1108,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Disparity / skew (option contracts)</t>
+          <t>Net premium ticks (call/put premium)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1126,7 +1118,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/option-contracts?limit</t>
+          <t>/api/stock/{t}/net-prem-ticks</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1142,12 +1134,12 @@
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 200 rows; {"delta": 0.240837729957301, "theta": -0.714354740675151, "gamma": 0.0589242960468416, "open_interes</t>
+          <t>AAPL: 248 rows; {"date": "2026-10-22", "call_volume": 3, "put_volume": 1, "call_volume_ask_side": 0, "call_volume_bi</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction, Unusual Activity</t>
+          <t>Claude, Meta, Unusual Activity</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1159,7 +1151,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>IV rank / implied volatility</t>
+          <t>Disparity / skew (option contracts)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1169,7 +1161,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/iv-rank</t>
+          <t>/api/stock/{t}/option-contracts?limit</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1185,12 +1177,12 @@
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 5 rows; {"close": "343.46", "date": "2026-10-16", "updated_at": "2026-10-16T22:35:01.364668Z", "volatility": "</t>
+          <t>AAPL: 200 rows; {"delta": 0.2098519710095163, "theta": -0.665797507508246, "gamma": 0.0547828939457017, "open_intere</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>IV Crush Check, Pre-Earnings Direction, Meta, Kimi, Gemini</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction, Unusual Activity</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1202,7 +1194,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Max pain / key option levels</t>
+          <t>IV rank / implied volatility</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1212,7 +1204,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/max-pain</t>
+          <t>/api/stock/{t}/iv-rank</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1228,12 +1220,12 @@
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 23 rows; {"close": "346.095", "open": "344.88", "expiry": "2026-10-23", "max_pain": "340", "next_upper_strike"</t>
+          <t>AAPL: 5 rows; {"close": "343.46", "date": "2026-10-16", "updated_at": "2026-10-16T22:35:01.364668Z", "volatility": "</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Pre-Earnings Direction, IV Crush Check</t>
+          <t>IV Crush Check, Pre-Earnings Direction, Meta, Kimi, Gemini</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1245,7 +1237,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Dark pool prints</t>
+          <t>Max pain / key option levels</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1255,7 +1247,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>/api/darkpool/{t}?limit</t>
+          <t>/api/stock/{t}/max-pain</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1271,12 +1263,12 @@
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 100 rows; {"size": 400, "ticker": "AAPL", "price": "346.1169", "volume": 15103132, "executed_at": "2026-10-22T</t>
+          <t>AAPL: 23 rows; {"close": "345.59", "open": "344.88", "expiry": "2026-10-23", "max_pain": "340", "next_upper_strike":</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
+          <t>Pre-Earnings Direction, IV Crush Check</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1288,7 +1280,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Volume price levels (dark-pool levels)</t>
+          <t>Dark pool prints</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1298,7 +1290,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>/api/stock/{t}/stock-volume-price-levels</t>
+          <t>/api/darkpool/{t}?limit</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1314,12 +1306,12 @@
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 19606 rows; {"price": 345.2057, "lit_vol": 0, "off_vol": 42}</t>
+          <t>AAPL: 100 rows; {"size": 460, "ticker": "AAPL", "price": "345.55", "volume": 16002694, "executed_at": "2026-10-22T16</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1331,7 +1323,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Short interest &amp; days-to-cover</t>
+          <t>Volume price levels (dark-pool levels)</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1341,7 +1333,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>/api/shorts/{t}/interest-float/v2</t>
+          <t>/api/stock/{t}/stock-volume-price-levels</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1357,12 +1349,12 @@
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 128 rows; {"symbol": "AAPL", "short_interest": 120763539, "market_date": "2026-09-30", "total_float": 14594180</t>
+          <t>AAPL: 20823 rows; {"price": 345.2057, "lit_vol": 0, "off_vol": 42}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
+          <t>Claude, Grok, Meta, ChatGPT</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1374,7 +1366,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Insider transactions (open-market buys)</t>
+          <t>Short interest &amp; days-to-cover</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1384,7 +1376,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>/api/insider/transactions?ticker_symbol&amp;limit</t>
+          <t>/api/shorts/{t}/interest-float/v2</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1400,12 +1392,12 @@
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 100 rows; {"id": "767c4106-4d41-4529-b0ad-78f88e29089b", "ticker": "AAPL", "amount": -1280, "transactions": 5,</t>
+          <t>AAPL: 128 rows; {"symbol": "AAPL", "short_interest": 120763539, "market_date": "2026-09-30", "total_float": 14594180</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro, Pre-Earnings Direction</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1417,7 +1409,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Insider flow summary</t>
+          <t>Insider transactions (open-market buys)</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1427,7 +1419,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>/api/insider/{t}</t>
+          <t>/api/insider/transactions?ticker_symbol&amp;limit</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1443,12 +1435,12 @@
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 50 rows; {"id": 167541, "name": "COOK TIMOTHY", "ticker": "AAPL", "display_name": "COOK TIMOTHY", "cik": "0001</t>
+          <t>AAPL: 100 rows; {"id": "767c4106-4d41-4529-b0ad-78f88e29089b", "ticker": "AAPL", "amount": -1280, "transactions": 5,</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1460,7 +1452,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Institutional ownership / big funds (13F)</t>
+          <t>Insider flow summary</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1470,7 +1462,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>/api/institution/{t}/ownership?limit</t>
+          <t>/api/insider/{t}</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1486,12 +1478,12 @@
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 100 rows; {"name": "BLACKROCK, INC.", "value": "336524794350", "units": "1162996939", "tags": [], "cik": "0002</t>
+          <t>AAPL: 50 rows; {"id": 167541, "name": "COOK TIMOTHY", "ticker": "AAPL", "display_name": "COOK TIMOTHY", "cik": "0001</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Claude, Claude Pro, Pre-Earnings Direction</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1503,7 +1495,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Analyst ratings / price targets</t>
+          <t>Institutional ownership / big funds (13F)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1513,7 +1505,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>/api/screener/analysts?ticker&amp;limit</t>
+          <t>/api/institution/{t}/ownership?limit</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1529,12 +1521,12 @@
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 20 rows; {"timestamp": "2026-10-20T18:01:21.000000Z", "ticker": "AAPL", "action": "maintained", "target": "283</t>
+          <t>AAPL: 100 rows; {"name": "BLACKROCK, INC.", "value": "336524794350", "units": "1162996939", "tags": [], "cik": "0002</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Grok, Kimi, Claude Pro</t>
+          <t>Claude, Claude Pro, Pre-Earnings Direction</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1546,7 +1538,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>News headlines</t>
+          <t>Analyst ratings (scored: Grok, ChatGPT, Kimi, Claude Pro)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1556,7 +1548,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>/api/news/headlines?ticker&amp;limit</t>
+          <t>/api/screener/analysts?ticker&amp;limit</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1572,12 +1564,12 @@
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 20 rows; {"meta": {}, "source": "Blockchain News", "created_at": "2026-10-22T12:20:14Z", "tags": [], "tickers"</t>
+          <t>AAPL: 20 rows; {"timestamp": "2026-10-20T18:01:21.000000Z", "ticker": "AAPL", "action": "maintained", "target": "283</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>News &amp; Sentiment</t>
+          <t>Grok, ChatGPT, Kimi, Claude Pro</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1589,7 +1581,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Earnings calendar / timing / implied move (pre-market)</t>
+          <t>News headlines</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1599,7 +1591,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>/api/earnings/premarket?date&amp;limit</t>
+          <t>/api/news/headlines?ticker&amp;limit</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1615,24 +1607,24 @@
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>54 rows; {"source": "company", "symbol": "PG", "country_code": "US", "full_name": "PROCTER &amp; GAMBLE", "sector"</t>
+          <t>AAPL: 20 rows; {"meta": {}, "source": "Blockchain News", "created_at": "2026-10-22T12:20:14Z", "tags": [], "tickers"</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Earnings Calendar, IV Crush Check, all models</t>
+          <t>News &amp; Sentiment</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>1/1</t>
+          <t>7/7</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Earnings calendar / timing / implied move (after-hours)</t>
+          <t>Earnings calendar / timing / implied move (pre-market)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1642,7 +1634,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>/api/earnings/afterhours?date&amp;limit</t>
+          <t>/api/earnings/premarket?date&amp;limit</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1658,7 +1650,7 @@
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>48 rows; {"source": "company", "symbol": "NEM", "country_code": "US", "full_name": "NEWMONT", "sector": "Basic</t>
+          <t>54 rows; {"source": "company", "symbol": "PG", "country_code": "US", "full_name": "PROCTER &amp; GAMBLE", "sector"</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1675,17 +1667,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Peer read-through: peers list</t>
+          <t>Earnings calendar / timing / implied move (after-hours)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Finnhub</t>
+          <t>Unusual Whales</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>/stock/peers?symbol</t>
+          <t>/api/earnings/afterhours?date&amp;limit</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1701,24 +1693,24 @@
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 11 rows; "AAPL"</t>
+          <t>48 rows; {"source": "company", "symbol": "NEM", "country_code": "US", "full_name": "NEWMONT", "sector": "Basic</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro</t>
+          <t>Earnings Calendar, IV Crush Check, all models</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>7/7</t>
+          <t>1/1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Analyst recommendations (Finnhub)</t>
+          <t>Peer read-through: peers list</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1728,7 +1720,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>/stock/recommendation?symbol</t>
+          <t>/stock/peers?symbol</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1744,12 +1736,12 @@
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 4 rows; {"symbol": "AAPL", "period": "2026-10-01", "strongBuy": 11, "buy": 20, "hold": 14, "sell": 3, "strongS</t>
+          <t>AAPL: 11 rows; "AAPL"</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Grok, Kimi, Claude Pro, ChatGPT</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi, Gemini, Claude Pro</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -1761,7 +1753,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Earnings surprise history (Finnhub)</t>
+          <t>Analyst recommendations (Finnhub)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1771,7 +1763,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>/stock/earnings?symbol</t>
+          <t>/stock/recommendation?symbol</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1787,12 +1779,12 @@
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 4 rows; {"symbol": "AAPL", "estimate": 1.9271, "actual": 1.91, "period": "2026-06-30", "surprise": -0.0171, "s</t>
+          <t>AAPL: 4 rows; {"symbol": "AAPL", "period": "2026-10-01", "strongBuy": 11, "buy": 20, "hold": 14, "sell": 3, "strongS</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Claude, Grok, Meta, ChatGPT, Kimi</t>
+          <t>Grok, Kimi, Claude Pro, ChatGPT</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -1804,7 +1796,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Price target (Finnhub)</t>
+          <t>Guidance hit-rate: 8Q EPS beat history (Finnhub)</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1814,33 +1806,33 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>/stock/price-target?symbol</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+          <t>/stock/earnings?symbol</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>403</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>7/7 calls failed (e.g. AAPL: You don't have access to this resource.)</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>AAPL: 4 rows; {"symbol": "AAPL", "estimate": 1.9271, "actual": 1.91, "period": "2026-06-30", "surprise": -0.0171, "s</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Grok, Kimi</t>
+          <t>Gemini</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>0/7</t>
+          <t>7/7</t>
         </is>
       </c>
     </row>
@@ -2023,134 +2015,91 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Earnings quality / Sloan accruals</t>
+          <t>VIX regime (app fallback value)</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Unusual Whales</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>NO DATA</t>
+          <t>kimi_service.vix_level()</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>no provider wired (scored neutral)</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>7.01 (VIXY 5-session change %)</t>
+        </is>
+      </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Gemini (Anas v2)</t>
+          <t>Kimi, Claude Pro</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>0/0</t>
+          <t>1/1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Guidance hit-rate history (12 qtrs)</t>
+          <t>BMO/AMC calendar timing (scored)</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Unusual Whales</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>NO DATA</t>
+          <t>/api/earnings/premarket|afterhours -&gt; report_time</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>no provider wired (scored neutral)</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr"/>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>PG: premarket -&gt; bias 1.0 (651/651 rows timed)</t>
+        </is>
+      </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Gemini (Anas v2)</t>
+          <t>Claude, Grok, Meta, ChatGPT, Kimi</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>0/0</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>BMO/AMC timing &amp; day-of-week</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>NO DATA</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>no scored input wired (neutral); calendar timing is read from the UW calendar rows</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Kimi (Anas v1 review), Claude (calendar), Grok, Meta, ChatGPT</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>0/0</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+          <t>651/651</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Run 2026-10-22 · tickers: AAPL, MSFT, NVDA, AMZN, TSLA, PG, AXP</t>
         </is>

</xml_diff>

<commit_message>
Low-data rule (<70% coverage), timing label-only, IBKR VIX primary, env-namespaced DB cache, All-in-One sheet reads each model tab, PED scan 166s->~10s
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data_Health_Check.xlsx
+++ b/Data_Health_Check.xlsx
@@ -661,7 +661,7 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 125 rows; {"source": "company", "report_date": "2026-11-02", "report_time": "postmarket", "ending_fiscal_quart</t>
+          <t>AAPL: 125 rows; {"source": "company", "report_time": "postmarket", "expected_move_perc": "0.04098141586521078892", "</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -747,7 +747,7 @@
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>AAPL: {"last_trade": {"price": "345.656", "time": 1792687345905, "vol": 15970483}, "market_time": "regular", "quote"</t>
+          <t>AAPL: {"last_trade": {"price": "345.71", "time": 1792691697639, "vol": 19776803}, "market_time": "regular", "quote":</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -790,7 +790,7 @@
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"last_trade": {"price": "763.32", "time": 1792687350082, "vol": 20547728}, "market_time": "regular", "quote":</t>
+          <t>{"last_trade": {"price": "762.96", "time": 1792691701651, "vol": 25170255}, "market_time": "regular", "quote":</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -876,7 +876,7 @@
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"last_trade": {"price": "17.5183", "time": 1792687345664, "vol": 3180656}, "market_time": "regular", "quote":</t>
+          <t>{"last_trade": {"price": "17.58", "time": 1792691703302, "vol": 3684956}, "market_time": "regular", "quote": {</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -919,7 +919,7 @@
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>62 rows; {"timestamp": "2026-10-22T07:30:00-04:00", "date": "2026-10-22", "net_call_premium": "-31513.0000", "</t>
+          <t>77 rows; {"timestamp": "2026-10-22T07:30:00-04:00", "date": "2026-10-22", "net_call_premium": "-31513.0000", "</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -962,7 +962,7 @@
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 50 rows; {"type": "put", "ticker": "AAPL", "iv": 0.31790407450507946, "created_at": "2026-10-22T16:42:20.70368</t>
+          <t>AAPL: 50 rows; {"type": "call", "ticker": "AAPL", "iv": 0.2870455207694094, "created_at": "2026-10-22T17:54:19.81223</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1005,7 +1005,7 @@
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 12 rows; {"theta": "-0.945558737799859", "cross_volume": 0, "delta": "-0.4455248061730525", "ticker_symbol": "</t>
+          <t>AAPL: 14 rows; {"no_side_volume": 0, "stock_price": "346.08", "expiry": "2026-10-23", "total_ask_changes": 17185, "d</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1091,7 +1091,7 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 1 rows; {"date": "2026-10-22", "call_volume": 354339, "put_volume": 304365, "call_volume_ask_side": 155182, "c</t>
+          <t>AAPL: 1 rows; {"date": "2026-10-22", "call_volume": 418164, "put_volume": 380615, "call_volume_ask_side": 183016, "c</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 248 rows; {"date": "2026-10-22", "call_volume": 3, "put_volume": 1, "call_volume_ask_side": 0, "call_volume_bi</t>
+          <t>AAPL: 321 rows; {"date": "2026-10-22", "call_volume": 3, "put_volume": 1, "call_volume_ask_side": 0, "call_volume_bi</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 200 rows; {"delta": 0.2098519710095163, "theta": -0.665797507508246, "gamma": 0.0547828939457017, "open_intere</t>
+          <t>AAPL: 200 rows; {"delta": 0.236690104377794, "theta": -0.751604268137119, "gamma": 0.0582407171666702, "open_interes</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1263,7 +1263,7 @@
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 23 rows; {"close": "345.59", "open": "344.88", "expiry": "2026-10-23", "max_pain": "340", "next_upper_strike":</t>
+          <t>AAPL: 23 rows; {"close": "346.0859", "open": "344.88", "expiry": "2026-10-23", "max_pain": "340", "next_upper_strike</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1306,7 +1306,7 @@
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 100 rows; {"size": 460, "ticker": "AAPL", "price": "345.55", "volume": 16002694, "executed_at": "2026-10-22T16</t>
+          <t>AAPL: 100 rows; {"size": 350, "ticker": "AAPL", "price": "346.06", "volume": 19886364, "executed_at": "2026-10-22T17</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1349,7 +1349,7 @@
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>AAPL: 20823 rows; {"price": 345.2057, "lit_vol": 0, "off_vol": 42}</t>
+          <t>AAPL: 23840 rows; {"price": 345.2057, "lit_vol": 0, "off_vol": 42}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1650,7 +1650,7 @@
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>54 rows; {"source": "company", "symbol": "PG", "country_code": "US", "full_name": "PROCTER &amp; GAMBLE", "sector"</t>
+          <t>54 rows; {"symbol": "PG", "source": "company", "country_code": "US", "full_name": "PROCTER &amp; GAMBLE", "sector"</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1693,7 +1693,7 @@
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>48 rows; {"source": "company", "symbol": "NEM", "country_code": "US", "full_name": "NEWMONT", "sector": "Basic</t>
+          <t>48 rows; {"symbol": "NEM", "source": "company", "country_code": "US", "full_name": "NEWMONT", "sector": "Basic</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2041,7 +2041,7 @@
       <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>7.01 (VIXY 5-session change %)</t>
+          <t>7.35 (VIXY 5-session change % (fallback))</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2084,7 +2084,7 @@
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>PG: premarket -&gt; bias 1.0 (651/651 rows timed)</t>
+          <t>PG: premarket -&gt; bias 1.0 (650/650 rows timed)</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>651/651</t>
+          <t>650/650</t>
         </is>
       </c>
     </row>

</xml_diff>